<commit_message>
increase max time wait
</commit_message>
<xml_diff>
--- a/Testkit_Q1_PRN222/Q11/TC1/Header.xlsx
+++ b/Testkit_Q1_PRN222/Q11/TC1/Header.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A856A5EF-22FE-4252-A633-4D9C6718F81A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6634FEC-509B-4328-A0E0-F4CE468ACA3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,9 +37,6 @@
     <t>Test Case ID</t>
   </si>
   <si>
-    <t>TC01</t>
-  </si>
-  <si>
     <t>Execution Date</t>
   </si>
   <si>
@@ -71,6 +68,9 @@
   </si>
   <si>
     <t>Type</t>
+  </si>
+  <si>
+    <t>TC1</t>
   </si>
 </sst>
 </file>
@@ -434,31 +434,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>2</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="3">
-        <v>20</v>
+        <v>120</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -479,31 +479,31 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" t="s">
         <v>8</v>
-      </c>
-      <c r="C1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="5"/>
       <c r="B2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>